<commit_message>
Atualiza dados e relatorio estatico
</commit_message>
<xml_diff>
--- a/Análise.xlsx
+++ b/Análise.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rafael/Documents/Projetos/proj_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7C6A8E-0D27-0646-AA02-A18D12C8E652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A2881B4-C0B3-5E4B-8D15-07F21BA13C53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{AE64DEAA-E857-E849-8ED4-9075A0D5982E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4532" uniqueCount="692">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4535" uniqueCount="693">
   <si>
     <t>SOBRAL</t>
   </si>
@@ -2110,6 +2110,9 @@
   </si>
   <si>
     <t>AIS</t>
+  </si>
+  <si>
+    <t>AIS 8, AIS 16, AIS 17, AIS 18, AIS 19, AIS 20, AIS 21</t>
   </si>
 </sst>
 </file>
@@ -2629,7 +2632,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2676,61 +2679,6 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="19">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF333333"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF333333"/>
-        <name val="Helvetica Neue"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Inherit"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2949,6 +2897,23 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Inherit"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2964,6 +2929,44 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <name val="Helvetica Neue"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <font>
@@ -3033,34 +3036,37 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{799F2E04-C2C5-284C-9BA4-A2232CAB350D}" name="Tabela5" displayName="Tabela5" ref="A1:E47" totalsRowShown="0" dataDxfId="18">
-  <autoFilter ref="A1:E47" xr:uid="{799F2E04-C2C5-284C-9BA4-A2232CAB350D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{799F2E04-C2C5-284C-9BA4-A2232CAB350D}" name="Tabela5" displayName="Tabela5" ref="A1:E48" totalsRowShown="0" dataDxfId="18">
+  <autoFilter ref="A1:E48" xr:uid="{799F2E04-C2C5-284C-9BA4-A2232CAB350D}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E48">
+    <sortCondition ref="D1:D48"/>
+  </sortState>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{887B31DD-663C-9445-936B-D1BCCBCD1136}" name="Quantidade de Escolas por Município" dataDxfId="17"/>
     <tableColumn id="2" xr3:uid="{A1740D3D-B389-894E-BD8F-8FBD5896BD58}" name="ESCOLAS" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{8F729B95-0637-BC4B-95A8-4494F5BD9374}" name="CRPM" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{D3D8B133-5742-A647-B4BA-AED3B495F607}" name="AIS" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{4060F7B6-BC58-4246-84C1-D46F87D1390D}" name="qtd_alunos" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{8F729B95-0637-BC4B-95A8-4494F5BD9374}" name="CRPM" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{D3D8B133-5742-A647-B4BA-AED3B495F607}" name="AIS" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{4060F7B6-BC58-4246-84C1-D46F87D1390D}" name="qtd_alunos" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9E3E37CB-73A3-F24E-AF9B-015DDF4CB31A}" name="Tabela1" displayName="Tabela1" ref="A1:K399" totalsRowShown="0" headerRowDxfId="2" dataDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9E3E37CB-73A3-F24E-AF9B-015DDF4CB31A}" name="Tabela1" displayName="Tabela1" ref="A1:K399" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="A1:K399" xr:uid="{9E3E37CB-73A3-F24E-AF9B-015DDF4CB31A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{5E5DF4A5-45C6-D24B-A745-C878F36EBD75}" name="MUNICIPIO" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{F0729342-B4AE-BC41-80D0-0723E70AC33B}" name="PARCELA_TERRITORIAL" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{3244A243-E44E-5949-85AB-70F8568A42C3}" name="RISP" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{14EEC560-DE97-DB4F-9E9E-57B14EAFABBD}" name="AIS_2026" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{9663A5A1-6B19-4641-AAA4-44F726A336D6}" name="CRPM" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{9DF37F3C-A5F7-F949-9452-F19CAA9049FA}" name="BPM" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{34ABAD3C-807D-D64F-8EA5-F49884EAC337}" name="DEL. SECCIONAL PCCE" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{FFF6AC92-8B0F-984F-8EDC-EE99870F0311}" name="CIRCUNSCRIÇÃO PCCE" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{DA17EBBA-3618-7942-B366-64C645C28CEA}" name="BBM" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{5718F28B-D7BB-AE4D-B805-486F9B534FC4}" name="CIA_BBM" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{6B7775C3-0AA1-6A4D-86B2-891D05A45BF2}" name="NÚCLEO PEFOCE" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{5E5DF4A5-45C6-D24B-A745-C878F36EBD75}" name="MUNICIPIO" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{F0729342-B4AE-BC41-80D0-0723E70AC33B}" name="PARCELA_TERRITORIAL" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{3244A243-E44E-5949-85AB-70F8568A42C3}" name="RISP" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{14EEC560-DE97-DB4F-9E9E-57B14EAFABBD}" name="AIS_2026" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{9663A5A1-6B19-4641-AAA4-44F726A336D6}" name="CRPM" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{9DF37F3C-A5F7-F949-9452-F19CAA9049FA}" name="BPM" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{34ABAD3C-807D-D64F-8EA5-F49884EAC337}" name="DEL. SECCIONAL PCCE" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{FFF6AC92-8B0F-984F-8EDC-EE99870F0311}" name="CIRCUNSCRIÇÃO PCCE" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{DA17EBBA-3618-7942-B366-64C645C28CEA}" name="BBM" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{5718F28B-D7BB-AE4D-B805-486F9B534FC4}" name="CIA_BBM" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{6B7775C3-0AA1-6A4D-86B2-891D05A45BF2}" name="NÚCLEO PEFOCE" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3383,7 +3389,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E5302BA-2BE3-EB44-9A21-698909D6DE66}">
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="34.33203125" customWidth="1"/>
@@ -3409,36 +3415,36 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>272</v>
+        <v>103</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="E2" s="1">
-        <v>2135</v>
+        <v>648</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>11</v>
+        <v>464</v>
       </c>
       <c r="B3" s="1">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>184</v>
+        <v>103</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="E3" s="1">
-        <v>1702</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -3460,95 +3466,95 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>324</v>
+        <v>198</v>
       </c>
       <c r="E5" s="1">
-        <v>1192</v>
+        <v>511</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B6" s="1">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>143</v>
+        <v>184</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>157</v>
+        <v>198</v>
       </c>
       <c r="E6" s="1">
-        <v>304</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="B7" s="1">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>84</v>
+        <v>184</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>335</v>
+        <v>198</v>
       </c>
       <c r="E7" s="1">
-        <v>846</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="B8" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>59</v>
+        <v>184</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>331</v>
+        <v>198</v>
       </c>
       <c r="E8" s="1">
-        <v>1671</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
-        <v>2</v>
+        <v>463</v>
       </c>
       <c r="B9" s="1">
         <v>8</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>334</v>
+        <v>74</v>
       </c>
       <c r="E9" s="1">
-        <v>490</v>
+        <v>456</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
-        <v>463</v>
+        <v>25</v>
       </c>
       <c r="B10" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>59</v>
@@ -3557,165 +3563,165 @@
         <v>74</v>
       </c>
       <c r="E10" s="1">
-        <v>456</v>
+        <v>438</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B11" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>184</v>
+        <v>59</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>198</v>
+        <v>74</v>
       </c>
       <c r="E11" s="1">
-        <v>511</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="1" t="s">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="B12" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>103</v>
+        <v>59</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>332</v>
+        <v>74</v>
       </c>
       <c r="E12" s="1">
-        <v>648</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="B13" s="1">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>84</v>
+        <v>173</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>83</v>
+        <v>324</v>
       </c>
       <c r="E13" s="1">
-        <v>521</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="1" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="B14" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>184</v>
+        <v>143</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>336</v>
+        <v>152</v>
       </c>
       <c r="E14" s="1">
-        <v>1011</v>
+        <v>264</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="1" t="s">
-        <v>464</v>
+        <v>32</v>
       </c>
       <c r="B15" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>103</v>
+        <v>143</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>332</v>
+        <v>152</v>
       </c>
       <c r="E15" s="1">
-        <v>279</v>
+        <v>215</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="1" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="B16" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>103</v>
+        <v>143</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>118</v>
+        <v>152</v>
       </c>
       <c r="E16" s="1">
-        <v>303</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="1">
         <v>1</v>
       </c>
-      <c r="B17" s="1">
-        <v>5</v>
-      </c>
       <c r="C17" s="1" t="s">
-        <v>84</v>
+        <v>143</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>334</v>
+        <v>152</v>
       </c>
       <c r="E17" s="1">
-        <v>264</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B18" s="1">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>103</v>
+        <v>184</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="E18" s="1">
-        <v>224</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" s="1">
         <v>5</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>59</v>
+        <v>184</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>74</v>
+        <v>336</v>
       </c>
       <c r="E19" s="1">
-        <v>438</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20" s="1">
         <v>4</v>
@@ -3724,35 +3730,35 @@
         <v>184</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>192</v>
+        <v>336</v>
       </c>
       <c r="E20" s="1">
-        <v>233</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B21" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>59</v>
+        <v>184</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>74</v>
+        <v>336</v>
       </c>
       <c r="E21" s="1">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="1" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="B22" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>184</v>
@@ -3761,151 +3767,151 @@
         <v>336</v>
       </c>
       <c r="E22" s="1">
-        <v>140</v>
+        <v>251</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="1" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="B23" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>84</v>
+        <v>184</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="E23" s="1">
-        <v>272</v>
+        <v>186</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="1" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="B24" s="1">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>184</v>
+        <v>143</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>336</v>
+        <v>157</v>
       </c>
       <c r="E24" s="1">
-        <v>228</v>
+        <v>304</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="1" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="B25" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>143</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="E25" s="1">
-        <v>264</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="1" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="B26" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>184</v>
+        <v>143</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>198</v>
+        <v>157</v>
       </c>
       <c r="E26" s="1">
-        <v>225</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="1" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="B27" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>143</v>
+        <v>84</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>152</v>
+        <v>249</v>
       </c>
       <c r="E27" s="1">
-        <v>215</v>
+        <v>375</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B28" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>184</v>
+        <v>84</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>336</v>
+        <v>83</v>
       </c>
       <c r="E28" s="1">
-        <v>251</v>
+        <v>521</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="1" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="B29" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>184</v>
+        <v>84</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>212</v>
+        <v>83</v>
       </c>
       <c r="E29" s="1">
-        <v>116</v>
+        <v>153</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B30" s="1">
         <v>2</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>184</v>
+        <v>59</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>227</v>
+        <v>66</v>
       </c>
       <c r="E30" s="1">
-        <v>215</v>
+        <v>94</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="1" t="s">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="B31" s="1">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>84</v>
@@ -3914,12 +3920,12 @@
         <v>335</v>
       </c>
       <c r="E31" s="1">
-        <v>233</v>
+        <v>846</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B32" s="1">
         <v>2</v>
@@ -3931,83 +3937,83 @@
         <v>335</v>
       </c>
       <c r="E32" s="1">
-        <v>96</v>
+        <v>233</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="B33" s="1">
         <v>2</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>184</v>
+        <v>84</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E33" s="1">
-        <v>186</v>
+        <v>96</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="1" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B34" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>66</v>
+        <v>335</v>
       </c>
       <c r="E34" s="1">
-        <v>94</v>
+        <v>179</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="1" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="B35" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>143</v>
+        <v>103</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>152</v>
+        <v>118</v>
       </c>
       <c r="E35" s="1">
-        <v>73</v>
+        <v>303</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B36" s="1">
         <v>2</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>74</v>
+        <v>118</v>
       </c>
       <c r="E36" s="1">
-        <v>161</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="1" t="s">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="B37" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>103</v>
@@ -4016,12 +4022,12 @@
         <v>118</v>
       </c>
       <c r="E37" s="1">
-        <v>148</v>
+        <v>81</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="1" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="B38" s="1">
         <v>2</v>
@@ -4030,163 +4036,180 @@
         <v>184</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="E38" s="1">
-        <v>207</v>
+        <v>116</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B39" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>59</v>
+        <v>184</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>331</v>
+        <v>227</v>
       </c>
       <c r="E39" s="1">
-        <v>236</v>
+        <v>215</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="1" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="B40" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>184</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="E40" s="1">
-        <v>130</v>
+        <v>233</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="1" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="B41" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>103</v>
+        <v>59</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>118</v>
+        <v>331</v>
       </c>
       <c r="E41" s="1">
-        <v>81</v>
+        <v>1671</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B42" s="1">
         <v>1</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>83</v>
+        <v>331</v>
       </c>
       <c r="E42" s="1">
-        <v>153</v>
+        <v>236</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="1" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B43" s="1">
-        <v>1</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>152</v>
+        <v>10</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>692</v>
       </c>
       <c r="E43" s="1">
-        <v>94</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="1" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="B44" s="1">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>157</v>
+        <v>272</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>692</v>
       </c>
       <c r="E44" s="1">
-        <v>22</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="1" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="B45" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>84</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>249</v>
+        <v>334</v>
       </c>
       <c r="E45" s="1">
-        <v>375</v>
+        <v>490</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46" s="1" t="s">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="B46" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>143</v>
+        <v>84</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>157</v>
+        <v>334</v>
       </c>
       <c r="E46" s="1">
-        <v>25</v>
+        <v>264</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" s="1" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="B47" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>84</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E47" s="1">
-        <v>179</v>
+        <v>272</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" s="1">
+        <v>5</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="E48" s="1">
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -4199,7 +4222,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7137C776-7244-3948-91D1-946AC9E356A1}">
-  <dimension ref="A1:L399"/>
+  <dimension ref="A1:K399"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
@@ -4212,7 +4235,7 @@
     <col min="11" max="11" width="23.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="18">
+    <row r="1" spans="1:11" ht="18">
       <c r="A1" s="5" t="s">
         <v>47</v>
       </c>
@@ -4246,9 +4269,8 @@
       <c r="K1" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="L1" s="6"/>
-    </row>
-    <row r="2" spans="1:12" ht="18">
+    </row>
+    <row r="2" spans="1:11" ht="18">
       <c r="A2" s="4" t="s">
         <v>20</v>
       </c>
@@ -4283,7 +4305,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="18">
+    <row r="3" spans="1:11" ht="18">
       <c r="A3" s="4" t="s">
         <v>340</v>
       </c>
@@ -4318,7 +4340,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="18">
+    <row r="4" spans="1:11" ht="18">
       <c r="A4" s="4" t="s">
         <v>341</v>
       </c>
@@ -4353,7 +4375,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="18">
+    <row r="5" spans="1:11" ht="18">
       <c r="A5" s="4" t="s">
         <v>342</v>
       </c>
@@ -4388,7 +4410,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="18">
+    <row r="6" spans="1:11" ht="18">
       <c r="A6" s="4" t="s">
         <v>343</v>
       </c>
@@ -4423,7 +4445,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="18">
+    <row r="7" spans="1:11" ht="18">
       <c r="A7" s="4" t="s">
         <v>344</v>
       </c>
@@ -4458,7 +4480,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="18">
+    <row r="8" spans="1:11" ht="18">
       <c r="A8" s="4" t="s">
         <v>345</v>
       </c>
@@ -4493,7 +4515,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="18">
+    <row r="9" spans="1:11" ht="18">
       <c r="A9" s="4" t="s">
         <v>346</v>
       </c>
@@ -4528,7 +4550,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="18">
+    <row r="10" spans="1:11" ht="18">
       <c r="A10" s="4" t="s">
         <v>347</v>
       </c>
@@ -4563,7 +4585,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="18">
+    <row r="11" spans="1:11" ht="18">
       <c r="A11" s="4" t="s">
         <v>348</v>
       </c>
@@ -4598,7 +4620,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="18">
+    <row r="12" spans="1:11" ht="18">
       <c r="A12" s="4" t="s">
         <v>36</v>
       </c>
@@ -4633,7 +4655,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="18">
+    <row r="13" spans="1:11" ht="18">
       <c r="A13" s="4" t="s">
         <v>349</v>
       </c>
@@ -4668,7 +4690,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="18">
+    <row r="14" spans="1:11" ht="18">
       <c r="A14" s="4" t="s">
         <v>350</v>
       </c>
@@ -4703,7 +4725,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="18">
+    <row r="15" spans="1:11" ht="18">
       <c r="A15" s="4" t="s">
         <v>351</v>
       </c>
@@ -4738,7 +4760,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="18">
+    <row r="16" spans="1:11" ht="18">
       <c r="A16" s="4" t="s">
         <v>352</v>
       </c>

</xml_diff>